<commit_message>
revised abstract and title
</commit_message>
<xml_diff>
--- a/Results/Sustainability gap.xlsx
+++ b/Results/Sustainability gap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Ongoing projects\Prospective LCA\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63C47D53-F476-4947-A5CF-2A6D89018083}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E471E9C-FF73-43A4-8A86-52B784A532C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025" xr2:uid="{9D5CE8AD-AD67-447A-B216-18105C8BC1BE}"/>
   </bookViews>
@@ -25,18 +25,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Methanol</t>
   </si>
   <si>
     <t>Hydrogen</t>
   </si>
+  <si>
+    <t>Ammonia</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -74,19 +80,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -407,198 +418,214 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="D1" s="3" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="G1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="3"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="A2" s="8">
         <v>2020</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="8">
         <v>2050</v>
       </c>
-      <c r="D2" s="2">
+      <c r="C2" s="7"/>
+      <c r="D2" s="8">
         <v>2020</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="8">
         <v>2050</v>
       </c>
-      <c r="G2" s="2">
+      <c r="F2" s="7"/>
+      <c r="G2" s="8">
         <v>2020</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="8">
         <v>2050</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>-0.84955861837746893</v>
-      </c>
-      <c r="B3" s="2">
-        <v>-1.320902128073866</v>
-      </c>
-      <c r="D3" s="2">
-        <v>2.399075197032861</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1.322298040883372</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0.85375564711232865</v>
-      </c>
-      <c r="H3" s="2">
-        <v>0.28589805137132751</v>
+      <c r="A3" s="4">
+        <v>-0.84955861837744795</v>
+      </c>
+      <c r="B3" s="4">
+        <v>-1.3209021280739359</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="4">
+        <v>2.3990751970328539</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1.3222980408833731</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="4">
+        <v>0.85375564711232665</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0.28589805137132768</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>-0.61823622845561277</v>
-      </c>
-      <c r="B4" s="2">
-        <v>-1.2475182875729991</v>
-      </c>
-      <c r="D4" s="2">
-        <v>4.063558420023198</v>
-      </c>
-      <c r="E4" s="2">
-        <v>1.850332406227821</v>
-      </c>
-      <c r="G4" s="2">
+      <c r="A4" s="4">
+        <v>-0.61823622845558535</v>
+      </c>
+      <c r="B4" s="4">
+        <v>-1.2475182875730371</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="4">
+        <v>4.0635584200231838</v>
+      </c>
+      <c r="E4" s="4">
+        <v>1.8503324062278219</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="4">
         <v>1.146704692771251</v>
       </c>
-      <c r="H4" s="2">
-        <v>0.37883209916837801</v>
+      <c r="H4" s="4">
+        <v>0.37883209916837851</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>0.76011638480268695</v>
-      </c>
-      <c r="B5" s="2">
-        <v>0.68341524385114316</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="A5" s="4">
+        <v>0.76011638480268706</v>
+      </c>
+      <c r="B5" s="4">
+        <v>0.68341524385114349</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="4">
         <v>11.07977878591611</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="4">
         <v>10.8619952521514</v>
       </c>
-      <c r="G5" s="2">
-        <v>2.697755753143285</v>
-      </c>
-      <c r="H5" s="2">
+      <c r="F5" s="5"/>
+      <c r="G5" s="4">
+        <v>2.6977557531432832</v>
+      </c>
+      <c r="H5" s="4">
         <v>2.5955168639584691</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="A6" s="4">
         <f>($A$5-A3)/$A$5*100</f>
-        <v>211.7669129837268</v>
-      </c>
-      <c r="B6" s="2">
+        <v>211.76691298372398</v>
+      </c>
+      <c r="B6" s="4">
         <f>($B$5-B3)/$B$5*100</f>
-        <v>293.27958220984254</v>
-      </c>
-      <c r="D6" s="2">
+        <v>293.27958220985266</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="4">
         <f>($D$5-D3)/$D$5*100</f>
-        <v>78.347264477135511</v>
-      </c>
-      <c r="E6" s="2">
+        <v>78.347264477135582</v>
+      </c>
+      <c r="E6" s="4">
         <f>($E$5-E3)/$E$5*100</f>
-        <v>87.826379866797794</v>
-      </c>
-      <c r="G6" s="2">
+        <v>87.826379866797765</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="4">
         <f>($G$5-G3)/$G$5*100</f>
-        <v>68.35311550656219</v>
-      </c>
-      <c r="H6" s="2">
+        <v>68.353115506562247</v>
+      </c>
+      <c r="H6" s="4">
         <f>($H$5-H3)/$H$5*100</f>
         <v>88.984927998683872</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="A7" s="4">
         <f>($A$5-A4)/$A$5*100</f>
-        <v>181.33441678356877</v>
-      </c>
-      <c r="B7" s="2">
+        <v>181.33441678356513</v>
+      </c>
+      <c r="B7" s="4">
         <f>($B$5-B4)/$B$5*100</f>
-        <v>282.54177073122543</v>
-      </c>
-      <c r="D7" s="2">
+        <v>282.54177073123094</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="4">
         <f>($D$5-D4)/$D$5*100</f>
-        <v>63.324552786301766</v>
-      </c>
-      <c r="E7" s="2">
+        <v>63.324552786301894</v>
+      </c>
+      <c r="E7" s="4">
         <f>($E$5-E4)/$E$5*100</f>
-        <v>82.965078116183761</v>
-      </c>
-      <c r="G7" s="2">
+        <v>82.965078116183733</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="4">
         <f>($G$5-G4)/$G$5*100</f>
-        <v>57.494124831902582</v>
-      </c>
-      <c r="H7" s="2">
+        <v>57.49412483190256</v>
+      </c>
+      <c r="H7" s="4">
         <f>($H$5-H4)/$H$5*100</f>
-        <v>85.404367645270682</v>
+        <v>85.404367645270668</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="A8" s="4">
         <f>AVERAGE(A6:A7)</f>
-        <v>196.55066488364778</v>
-      </c>
-      <c r="B8" s="2">
+        <v>196.55066488364457</v>
+      </c>
+      <c r="B8" s="4">
         <f>AVERAGE(B6:B7)</f>
-        <v>287.91067647053399</v>
-      </c>
-      <c r="D8" s="2">
+        <v>287.91067647054183</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="4">
         <f>AVERAGE(D6:D7)</f>
-        <v>70.835908631718638</v>
-      </c>
-      <c r="E8" s="2">
+        <v>70.835908631718738</v>
+      </c>
+      <c r="E8" s="4">
         <f>AVERAGE(E6:E7)</f>
-        <v>85.395728991490785</v>
-      </c>
-      <c r="G8" s="2">
+        <v>85.395728991490756</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="4">
         <f>AVERAGE(G6:G7)</f>
-        <v>62.923620169232386</v>
-      </c>
-      <c r="H8" s="2">
+        <v>62.923620169232407</v>
+      </c>
+      <c r="H8" s="4">
         <f>AVERAGE(H6:H7)</f>
         <v>87.19464782197727</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <f>(B8-A8)/A8*100</f>
-        <v>46.481659902279468</v>
+        <v>46.481659902285855</v>
       </c>
       <c r="C9" s="1"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="4">
+      <c r="D9" s="3"/>
+      <c r="E9" s="2">
         <f>(E8-D8)/D8*100</f>
-        <v>20.554293212316619</v>
+        <v>20.554293212316409</v>
       </c>
       <c r="F9" s="1"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="4">
+      <c r="G9" s="3"/>
+      <c r="H9" s="2">
         <f>(H8-G8)/G8*100</f>
-        <v>38.57220482144578</v>
+        <v>38.57220482144573</v>
       </c>
       <c r="I9" s="1"/>
-      <c r="J9" s="4">
+      <c r="J9" s="2">
         <f>AVERAGE(B9:H9)</f>
-        <v>35.202719312013954</v>
+        <v>35.202719312016001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>